<commit_message>
feat: update export people template to include registered date + remove sample data
</commit_message>
<xml_diff>
--- a/src/backend/resources/templates/export_people_template.xlsx
+++ b/src/backend/resources/templates/export_people_template.xlsx
@@ -1,39 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11207"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/daniel/Development/micropowermanager/src/backend/resources/templates/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCF1888C-9813-2E42-B5A2-D572205B0E55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29420" windowHeight="15460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="11">
   <si>
     <t>Title</t>
   </si>
@@ -44,9 +26,15 @@
     <t>Surname</t>
   </si>
   <si>
+    <t>Registered Date</t>
+  </si>
+  <si>
     <t>Birth Date</t>
   </si>
   <si>
+    <t>Gender</t>
+  </si>
+  <si>
     <t>Email</t>
   </si>
   <si>
@@ -60,88 +48,22 @@
   </si>
   <si>
     <t>Agent Name</t>
-  </si>
-  <si>
-    <t>Dr.</t>
-  </si>
-  <si>
-    <t>Sven</t>
-  </si>
-  <si>
-    <t>Predovic</t>
-  </si>
-  <si>
-    <t>2014-06-11</t>
-  </si>
-  <si>
-    <t>Female</t>
-  </si>
-  <si>
-    <t>beatty.tad@example.com</t>
-  </si>
-  <si>
-    <t>+14587089684</t>
-  </si>
-  <si>
-    <t>Mafia Village</t>
-  </si>
-  <si>
-    <t>40c6ff72-545a-3821-81fd-2f701aa7f7fb</t>
-  </si>
-  <si>
-    <t>Nikki</t>
-  </si>
-  <si>
-    <t>Mr.</t>
-  </si>
-  <si>
-    <t>John</t>
-  </si>
-  <si>
-    <t>Doe</t>
-  </si>
-  <si>
-    <t>1985-01-01</t>
-  </si>
-  <si>
-    <t>Male</t>
-  </si>
-  <si>
-    <t>john.doe@example.com</t>
-  </si>
-  <si>
-    <t>+1234567890</t>
-  </si>
-  <si>
-    <t>Sun City</t>
-  </si>
-  <si>
-    <t>ABC123456789</t>
-  </si>
-  <si>
-    <t>Jane Smith</t>
-  </si>
-  <si>
-    <t>Gender</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -166,22 +88,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <tableStyles defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotTableStyle1"/>
 </styleSheet>
 </file>
 
@@ -469,11 +383,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xml:space="preserve" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr defaultRowHeight="14.4" defaultColWidth="9" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -486,90 +403,31 @@
       <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="F1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
       <c r="G1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
         <v>9</v>
       </c>
-      <c r="B2" t="s">
+      <c r="K1" t="s">
         <v>10</v>
-      </c>
-      <c r="C2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G2" t="s">
-        <v>15</v>
-      </c>
-      <c r="H2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I2" t="s">
-        <v>17</v>
-      </c>
-      <c r="J2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C3" t="s">
-        <v>21</v>
-      </c>
-      <c r="D3" t="s">
-        <v>22</v>
-      </c>
-      <c r="E3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F3" t="s">
-        <v>24</v>
-      </c>
-      <c r="G3" t="s">
-        <v>25</v>
-      </c>
-      <c r="H3" t="s">
-        <v>26</v>
-      </c>
-      <c r="I3" t="s">
-        <v>27</v>
-      </c>
-      <c r="J3" t="s">
-        <v>28</v>
       </c>
     </row>
   </sheetData>
+  <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: update export people template to include registered date + remove sample data (#1556)
</commit_message>
<xml_diff>
--- a/src/backend/resources/templates/export_people_template.xlsx
+++ b/src/backend/resources/templates/export_people_template.xlsx
@@ -1,39 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11207"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/daniel/Development/micropowermanager/src/backend/resources/templates/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCF1888C-9813-2E42-B5A2-D572205B0E55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29420" windowHeight="15460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="11">
   <si>
     <t>Title</t>
   </si>
@@ -44,9 +26,15 @@
     <t>Surname</t>
   </si>
   <si>
+    <t>Registered Date</t>
+  </si>
+  <si>
     <t>Birth Date</t>
   </si>
   <si>
+    <t>Gender</t>
+  </si>
+  <si>
     <t>Email</t>
   </si>
   <si>
@@ -60,88 +48,22 @@
   </si>
   <si>
     <t>Agent Name</t>
-  </si>
-  <si>
-    <t>Dr.</t>
-  </si>
-  <si>
-    <t>Sven</t>
-  </si>
-  <si>
-    <t>Predovic</t>
-  </si>
-  <si>
-    <t>2014-06-11</t>
-  </si>
-  <si>
-    <t>Female</t>
-  </si>
-  <si>
-    <t>beatty.tad@example.com</t>
-  </si>
-  <si>
-    <t>+14587089684</t>
-  </si>
-  <si>
-    <t>Mafia Village</t>
-  </si>
-  <si>
-    <t>40c6ff72-545a-3821-81fd-2f701aa7f7fb</t>
-  </si>
-  <si>
-    <t>Nikki</t>
-  </si>
-  <si>
-    <t>Mr.</t>
-  </si>
-  <si>
-    <t>John</t>
-  </si>
-  <si>
-    <t>Doe</t>
-  </si>
-  <si>
-    <t>1985-01-01</t>
-  </si>
-  <si>
-    <t>Male</t>
-  </si>
-  <si>
-    <t>john.doe@example.com</t>
-  </si>
-  <si>
-    <t>+1234567890</t>
-  </si>
-  <si>
-    <t>Sun City</t>
-  </si>
-  <si>
-    <t>ABC123456789</t>
-  </si>
-  <si>
-    <t>Jane Smith</t>
-  </si>
-  <si>
-    <t>Gender</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -166,22 +88,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <tableStyles defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotTableStyle1"/>
 </styleSheet>
 </file>
 
@@ -469,11 +383,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xml:space="preserve" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr defaultRowHeight="14.4" defaultColWidth="9" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -486,90 +403,31 @@
       <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="F1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
       <c r="G1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
         <v>9</v>
       </c>
-      <c r="B2" t="s">
+      <c r="K1" t="s">
         <v>10</v>
-      </c>
-      <c r="C2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G2" t="s">
-        <v>15</v>
-      </c>
-      <c r="H2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I2" t="s">
-        <v>17</v>
-      </c>
-      <c r="J2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C3" t="s">
-        <v>21</v>
-      </c>
-      <c r="D3" t="s">
-        <v>22</v>
-      </c>
-      <c r="E3" t="s">
-        <v>23</v>
-      </c>
-      <c r="F3" t="s">
-        <v>24</v>
-      </c>
-      <c r="G3" t="s">
-        <v>25</v>
-      </c>
-      <c r="H3" t="s">
-        <v>26</v>
-      </c>
-      <c r="I3" t="s">
-        <v>27</v>
-      </c>
-      <c r="J3" t="s">
-        <v>28</v>
       </c>
     </row>
   </sheetData>
+  <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(export): add appliance, cluster, and site info to person export
- Include appliance names linked to each person's devices, accounting for SolarHomeSystem and EBike types
- Add cluster name and mini-grid (site) name derived from the primary address city
</commit_message>
<xml_diff>
--- a/src/backend/resources/templates/export_people_template.xlsx
+++ b/src/backend/resources/templates/export_people_template.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView windowWidth="28000" windowHeight="15760"/>
+    <workbookView windowHeight="17140"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>Title</t>
   </si>
@@ -65,7 +65,19 @@
     <t>Device Serial</t>
   </si>
   <si>
+    <t>Appliance Name</t>
+  </si>
+  <si>
+    <t>Cluster Name</t>
+  </si>
+  <si>
+    <t>Site Name (MiniGrid Name)</t>
+  </si>
+  <si>
     <t>Agent Name</t>
+  </si>
+  <si>
+    <t>Last Payment</t>
   </si>
 </sst>
 </file>
@@ -696,7 +708,7 @@
     <cellStyle name="Percent" xfId="3" builtinId="5"/>
     <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
     <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Hyperlink" xfId="6" builtinId="8"/>
+    <cellStyle name="Link" xfId="6" builtinId="8"/>
     <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
     <cellStyle name="Note" xfId="8" builtinId="10"/>
     <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
@@ -1034,16 +1046,29 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:Q1"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
-    <col min="9" max="9" width="7.2890625" customWidth="1"/>
-    <col min="11" max="11" width="20.5703125" customWidth="1"/>
-    <col min="12" max="12" width="11.1953125" customWidth="1"/>
-    <col min="13" max="13" width="10.671875" customWidth="1"/>
+    <col min="1" max="1" width="4.75" customWidth="1"/>
+    <col min="2" max="2" width="6.125" customWidth="1"/>
+    <col min="3" max="3" width="8.5625" customWidth="1"/>
+    <col min="4" max="4" width="14.5625" customWidth="1"/>
+    <col min="5" max="5" width="9.375" customWidth="1"/>
+    <col min="6" max="6" width="7.3125" customWidth="1"/>
+    <col min="7" max="7" width="5.75" customWidth="1"/>
+    <col min="8" max="8" width="6.5625" customWidth="1"/>
+    <col min="9" max="9" width="4.5625" customWidth="1"/>
+    <col min="10" max="10" width="6.1875" customWidth="1"/>
+    <col min="11" max="11" width="32.3125" customWidth="1"/>
+    <col min="12" max="12" width="11.8125" customWidth="1"/>
+    <col min="13" max="13" width="14.9375" customWidth="1"/>
+    <col min="14" max="14" width="12.4375" customWidth="1"/>
+    <col min="15" max="15" width="24" customWidth="1"/>
+    <col min="16" max="16" width="11.375" customWidth="1"/>
+    <col min="17" max="17" width="12.5625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:17">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1082,6 +1107,18 @@
       </c>
       <c r="M1" t="s">
         <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>